<commit_message>
Before removing unused variable
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Atominos Consulting\Documents\UiPath\Gulf Drug Process\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E72017-9011-4903-A936-A8399B173036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D407B5D1-C988-46E7-9BBE-51F98F9C0ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -459,7 +459,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -478,7 +478,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -898,7 +897,7 @@
       <c r="A8" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" t="s">
         <v>119</v>
       </c>
       <c r="C8" s="4"/>
@@ -916,7 +915,7 @@
       <c r="A10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" t="s">
         <v>120</v>
       </c>
       <c r="C10" s="4"/>

</xml_diff>